<commit_message>
feat: fase implementacion y pruebas
</commit_message>
<xml_diff>
--- a/docs/ciclo 2/Acta de reunion ciclo 2.xlsx
+++ b/docs/ciclo 2/Acta de reunion ciclo 2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{567AD540-3ECF-4153-80DA-90F419057D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E9F48AA-C9AF-4F51-9455-65E51FF156F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="11040" activeTab="1" xr2:uid="{62DC227A-B2C0-4B2D-82A6-53B37F2213DD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{62DC227A-B2C0-4B2D-82A6-53B37F2213DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Ciclo 1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="46">
   <si>
     <t>Acta de Reuniones</t>
   </si>
@@ -177,6 +177,19 @@
   </si>
   <si>
     <t>Se realizo la reunion grupal con el proposito de distribuir los casos de uso para el segundo ciclo a trabaja, a su vez actualizando los documentos correspondientes a especificacion de requerimientos SRS, modelo de casos de uso, modelo de dominio, plan de calidad, plan de administracion y requerimientos y EDT</t>
+  </si>
+  <si>
+    <t>Se realizo la reunion con el proposito de modificar y perfeccionar los diferentes diagramas realizados en la fase 1 para agregar o extender funcionalidades para el ciclo 2</t>
+  </si>
+  <si>
+    <t>Se realizo la reunion con el proposito de diligenciar y distribuir los documentos correspondientes a la fase de implementacion y pruebas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documentacion Script fase de diseño del ciclo 2
+</t>
+  </si>
+  <si>
+    <t>Documentacion Script fase de implementacion y pruebas para el ciclo 2</t>
   </si>
 </sst>
 </file>
@@ -256,7 +269,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -279,11 +292,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -634,34 +650,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
@@ -1050,7 +1066,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A942043F-F080-4F69-8AC5-CB25BD518FCB}">
-  <dimension ref="B1:M5"/>
+  <dimension ref="B1:M7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.5546875" style="1"/>
@@ -1070,34 +1086,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
@@ -1156,12 +1172,12 @@
       <c r="G4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
     </row>
     <row r="5" spans="2:13" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="3">
@@ -1182,12 +1198,52 @@
       <c r="G5" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+    </row>
+    <row r="6" spans="2:13" ht="73.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="3">
+        <v>3</v>
+      </c>
+      <c r="C6" s="4">
+        <v>45971</v>
+      </c>
+      <c r="D6" s="5">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="E6" s="5">
+        <v>0.875</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+    </row>
+    <row r="7" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F7" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>